<commit_message>
Birth years for eleven more players from school and college records
Second search pass over the 72 players still without a year. Found class
years for Gramley, Troutman, Oehrle, Yofan, Grzegorczyk, Wymard, Koerbel,
Rathfon, Pepe and Cordaro at Longue Vue and Frank Fuhrer IV at the Field
Club, all stored as approximate. The rest are listed in the file as
searched with nothing found. Spreadsheet for the clubs rebuilt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -1102,17 +1102,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr"/>
-      <c r="E21" s="7" t="n"/>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1999</v>
+      </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Shady Side Academy senior in fall 2017</t>
+        </is>
+      </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -5792,17 +5802,27 @@
           <t>2013–2018</t>
         </is>
       </c>
-      <c r="D155" s="6" t="inlineStr"/>
-      <c r="E155" s="7" t="n"/>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="n">
+        <v>1997</v>
+      </c>
       <c r="F155" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G155" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G155" s="8" t="inlineStr">
+        <is>
+          <t>Pittsburgh entrant in 2014 U.S. Junior Amateur qualifying (under 19); uncertain by a year or two</t>
+        </is>
+      </c>
       <c r="H155" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6132,17 +6152,27 @@
           <t>2014–2015</t>
         </is>
       </c>
-      <c r="D166" s="6" t="inlineStr"/>
-      <c r="E166" s="7" t="n"/>
+      <c r="D166" s="6" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="E166" s="7" t="n">
+        <v>1994</v>
+      </c>
       <c r="F166" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G166" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G166" s="8" t="inlineStr">
+        <is>
+          <t>Shady Side Academy; senior on the South Carolina golf roster 2015-16</t>
+        </is>
+      </c>
       <c r="H166" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6162,17 +6192,27 @@
           <t>2022–2023</t>
         </is>
       </c>
-      <c r="D167" s="6" t="inlineStr"/>
-      <c r="E167" s="7" t="n"/>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="n">
+        <v>2000</v>
+      </c>
       <c r="F167" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G167" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G167" s="8" t="inlineStr">
+        <is>
+          <t>Shaler graduate; Findlay golf, senior in 2023; uncertain by a year or two</t>
+        </is>
+      </c>
       <c r="H167" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6252,17 +6292,27 @@
           <t>2021–2025</t>
         </is>
       </c>
-      <c r="D170" s="6" t="inlineStr"/>
-      <c r="E170" s="7" t="n"/>
+      <c r="D170" s="6" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="E170" s="7" t="n">
+        <v>1990</v>
+      </c>
       <c r="F170" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G170" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G170" s="8" t="inlineStr">
+        <is>
+          <t>Deer Lakes; Penn State Behrend golf 2009-11</t>
+        </is>
+      </c>
       <c r="H170" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6372,17 +6422,27 @@
           <t>2019–2025</t>
         </is>
       </c>
-      <c r="D174" s="6" t="inlineStr"/>
-      <c r="E174" s="7" t="n"/>
+      <c r="D174" s="6" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="E174" s="7" t="n">
+        <v>2003</v>
+      </c>
       <c r="F174" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G174" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G174" s="8" t="inlineStr">
+        <is>
+          <t>Fox Chapel HS junior in fall 2019 (WPIAL 3A, T3)</t>
+        </is>
+      </c>
       <c r="H174" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6432,17 +6492,27 @@
           <t>2009–2013</t>
         </is>
       </c>
-      <c r="D176" s="6" t="inlineStr"/>
-      <c r="E176" s="7" t="n"/>
+      <c r="D176" s="6" t="inlineStr">
+        <is>
+          <t>1986</t>
+        </is>
+      </c>
+      <c r="E176" s="7" t="n">
+        <v>1986</v>
+      </c>
       <c r="F176" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G176" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G176" s="8" t="inlineStr">
+        <is>
+          <t>Serra Catholic; senior on the Marshall golf roster 2007-08</t>
+        </is>
+      </c>
       <c r="H176" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6462,17 +6532,27 @@
           <t>2009–2014</t>
         </is>
       </c>
-      <c r="D177" s="6" t="inlineStr"/>
-      <c r="E177" s="7" t="n"/>
+      <c r="D177" s="6" t="inlineStr">
+        <is>
+          <t>1983</t>
+        </is>
+      </c>
+      <c r="E177" s="7" t="n">
+        <v>1983</v>
+      </c>
       <c r="F177" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G177" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G177" s="8" t="inlineStr">
+        <is>
+          <t>Allegheny College class of 2005 (athletics hall of fame)</t>
+        </is>
+      </c>
       <c r="H177" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6552,17 +6632,27 @@
           <t>2020–2025</t>
         </is>
       </c>
-      <c r="D180" s="6" t="inlineStr"/>
-      <c r="E180" s="7" t="n"/>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="E180" s="7" t="n">
+        <v>2003</v>
+      </c>
       <c r="F180" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G180" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G180" s="8" t="inlineStr">
+        <is>
+          <t>Shady Side Academy sophomore in fall 2018 (IPSL medalist)</t>
+        </is>
+      </c>
       <c r="H180" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6732,17 +6822,27 @@
           <t>2023–2025</t>
         </is>
       </c>
-      <c r="D186" s="6" t="inlineStr"/>
-      <c r="E186" s="7" t="n"/>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="E186" s="7" t="n">
+        <v>2001</v>
+      </c>
       <c r="F186" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G186" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
+          <t>Pine-Richland golfer at the 2018 PIAA championship; class year not found, uncertain</t>
+        </is>
+      </c>
       <c r="H186" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6762,17 +6862,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D187" s="6" t="inlineStr"/>
-      <c r="E187" s="7" t="n"/>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="E187" s="7" t="n">
+        <v>2004</v>
+      </c>
       <c r="F187" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G187" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G187" s="8" t="inlineStr">
+        <is>
+          <t>Fox Chapel HS junior in fall 2020</t>
+        </is>
+      </c>
       <c r="H187" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6851,13 +6961,13 @@
         <v>34</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -6917,13 +7027,13 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -6939,13 +7049,13 @@
         <v>90</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Field Club birth dates from Tommy; name Dunlap and Banks on the sheets
DJ Claus gets his full date, Matt Dunlap and Dom Fazio theirs, and Banks,
Frohlich and Maher an approximate year from an age or class year. Dunlap
and Banks, surname-only on the 2025 sheet, are pinned in players.yaml as
Matt Dunlap and Ryan Banks. Spreadsheet rebuilt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Banks</t>
+          <t>Ryan Banks</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -592,17 +592,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="7" t="n"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>1990</v>
+      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Age 36 in Oct 2026 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -762,7 +772,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Jun 1983</t>
+          <t>15 Jun 1983</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -775,7 +785,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Field Club age roster, Aug 2025 (month and year only)</t>
+          <t>Field Club age roster, Aug 2025; full date from Tommy Leech, Oct 2026</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr"/>
@@ -860,7 +870,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Dunlap</t>
+          <t>Matt Dunlap</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -868,19 +878,25 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="7" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>7 Dec 1993</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1993</v>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr"/>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Please add</t>
-        </is>
-      </c>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Tommy Leech, Oct 2026</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -970,19 +986,25 @@
           <t>2024–2025</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="7" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>24 May 1993</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1993</v>
+      </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr"/>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Please add</t>
-        </is>
-      </c>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Tommy Leech, Oct 2026</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1036,17 +1058,27 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="7" t="n"/>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>2007</v>
+      </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>High school class of 2025 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -1322,17 +1354,27 @@
           <t>2014–2015</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr"/>
-      <c r="E27" s="7" t="n"/>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>1994</v>
+      </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>High school class of 2012 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6958,16 +7000,16 @@
         <v>41</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -7046,16 +7088,16 @@
         <v>182</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Three more rough birth-year estimates; note the third search pass
Will Betts, James Braham (probably Jimmy Brahm, the former Fox Chapel
assistant pro) and Gus Schroeder Jr. get approximate years with the
uncertainty spelled out in the source. A pass over high-school and
college sports sites found nothing for the other 53 names; the file
says so.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -2304,17 +2304,27 @@
           <t>2015</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr"/>
-      <c r="E54" s="7" t="n"/>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>1977</v>
+      </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>Probably Jimmy Brahm, PGA, former Fox Chapel assistant pro: Slippery Rock graduate who entered the golf business in 2000; identity and year both uncertain</t>
+        </is>
+      </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -3466,17 +3476,27 @@
           <t>2007–2021</t>
         </is>
       </c>
-      <c r="D87" s="6" t="inlineStr"/>
-      <c r="E87" s="7" t="n"/>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="n">
+        <v>1970</v>
+      </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G87" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Gus Schroeder Jr., Schroeder Industries president since 2005; rough estimate, father (also Gus, b. c. 1940) died c. 2000</t>
+        </is>
+      </c>
       <c r="H87" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -5694,17 +5714,27 @@
           <t>2008–2025</t>
         </is>
       </c>
-      <c r="D150" s="6" t="inlineStr"/>
-      <c r="E150" s="7" t="n"/>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="E150" s="7" t="n">
+        <v>1994</v>
+      </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G150" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="G150" s="8" t="inlineStr">
+        <is>
+          <t>A William Betts of Leechburg was a Hartford golf senior in 2015-16; if the same man he was 14 at his 2008 debut, so uncertain</t>
+        </is>
+      </c>
       <c r="H150" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -7025,13 +7055,13 @@
         <v>16</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>3</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -7069,13 +7099,13 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -7091,13 +7121,13 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Will Betts: born c. 1993, from Tommy (Fox Chapel freshman 2007)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -5716,11 +5716,11 @@
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="E150" s="7" t="n">
-        <v>1994</v>
+        <v>1993</v>
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>A William Betts of Leechburg was a Hartford golf senior in 2015-16; if the same man he was 14 at his 2008 debut, so uncertain</t>
+          <t>Fox Chapel HS freshman in 2007, then prep school, class of 2011/12 (Tommy Leech); Hartford golf senior 2015-16</t>
         </is>
       </c>
       <c r="H150" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Age bands: store "50+"-style answers, show roster by band
A captain's "he's 50+" is a band, not a year, so birthdates.yaml takes
`band` + `asOf` instead of `born` and players gain age_band /
age_band_year (migration 0003). src/lib/ages.ts defines the bands
(under 25, 25-29, 30-39, 40-49, 50+) and shifts a stored band to another
season. Leaderboards get a roster-by-band table where band-only players
count as "+n" in the lowest band they could be in; the player page shows
"age 50+ in 2026". Colville, McBride and Crawford stored as 50+.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Birth dates'!$A$5:$H$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Birth dates'!$A$5:$I$187</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H187"/>
+  <dimension ref="A1:I187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -508,9 +508,10 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -562,15 +563,20 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
+          <t>Age band (2026)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Where it came from</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Notes for the club</t>
         </is>
@@ -602,15 +608,20 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Age 36 in Oct 2026 (Tommy Leech)</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -642,15 +653,20 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -678,15 +694,20 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -714,15 +735,20 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -742,13 +768,14 @@
       </c>
       <c r="D10" s="6" t="inlineStr"/>
       <c r="E10" s="7" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr"/>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -780,15 +807,20 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025; full date from Tommy Leech, Oct 2026</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -816,15 +848,20 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -852,15 +889,20 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -888,15 +930,20 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Tommy Leech, Oct 2026</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -924,15 +971,20 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -960,15 +1012,20 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -996,15 +1053,20 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>Tommy Leech, Oct 2026</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr"/>
+      <c r="I17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1032,15 +1094,20 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1068,15 +1135,20 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>High school class of 2025 (Tommy Leech)</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -1108,15 +1180,20 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr"/>
+      <c r="I20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1144,15 +1221,20 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>Shady Side Academy senior in fall 2017</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -1184,15 +1266,20 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr"/>
+      <c r="I22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1220,15 +1307,20 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1256,15 +1348,20 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1292,15 +1389,20 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1328,15 +1430,20 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1364,15 +1471,20 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
         <is>
           <t>High school class of 2012 (Tommy Leech)</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -1404,15 +1516,20 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1440,15 +1557,20 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr"/>
+      <c r="I29" s="8" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1476,15 +1598,20 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr"/>
+      <c r="I30" s="8" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1512,15 +1639,20 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr"/>
+      <c r="I31" s="8" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1548,15 +1680,20 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr"/>
+      <c r="I32" s="8" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1584,15 +1721,20 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr"/>
+      <c r="I33" s="8" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1620,15 +1762,20 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G34" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr"/>
+      <c r="I34" s="8" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1656,15 +1803,20 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr"/>
+      <c r="I35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1692,15 +1844,20 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr"/>
+      <c r="I36" s="8" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1728,15 +1885,20 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr"/>
+      <c r="I37" s="8" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1764,15 +1926,20 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr"/>
+      <c r="I38" s="8" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -1800,15 +1967,20 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H39" s="8" t="inlineStr"/>
+      <c r="I39" s="8" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -1836,15 +2008,20 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G40" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr"/>
+      <c r="I40" s="8" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -1872,15 +2049,20 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G41" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr"/>
+      <c r="I41" s="8" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -1908,15 +2090,20 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G42" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr"/>
+      <c r="I42" s="8" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -1944,15 +2131,20 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H43" s="8" t="inlineStr"/>
+      <c r="I43" s="8" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -1980,15 +2172,20 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr"/>
+      <c r="I44" s="8" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -2016,15 +2213,20 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr"/>
+      <c r="I45" s="8" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2052,15 +2254,20 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
         <is>
           <t>Field Club age roster, Aug 2025 (month and year only)</t>
         </is>
       </c>
-      <c r="H46" s="8" t="inlineStr"/>
+      <c r="I46" s="8" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -2080,13 +2287,14 @@
       </c>
       <c r="D47" s="6" t="inlineStr"/>
       <c r="E47" s="7" t="n"/>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr"/>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="H47" s="8" t="inlineStr"/>
+      <c r="I47" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2110,13 +2318,14 @@
       </c>
       <c r="D48" s="6" t="inlineStr"/>
       <c r="E48" s="7" t="n"/>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr"/>
-      <c r="H48" s="8" t="inlineStr">
+      <c r="H48" s="8" t="inlineStr"/>
+      <c r="I48" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2140,13 +2349,14 @@
       </c>
       <c r="D49" s="6" t="inlineStr"/>
       <c r="E49" s="7" t="n"/>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G49" s="8" t="inlineStr"/>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="H49" s="8" t="inlineStr"/>
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2170,13 +2380,14 @@
       </c>
       <c r="D50" s="6" t="inlineStr"/>
       <c r="E50" s="7" t="n"/>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G50" s="8" t="inlineStr"/>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="H50" s="8" t="inlineStr"/>
+      <c r="I50" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2200,13 +2411,14 @@
       </c>
       <c r="D51" s="6" t="inlineStr"/>
       <c r="E51" s="7" t="n"/>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G51" s="8" t="inlineStr"/>
-      <c r="H51" s="8" t="inlineStr">
+      <c r="H51" s="8" t="inlineStr"/>
+      <c r="I51" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2238,15 +2450,20 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G52" s="8" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel HS class of 2028 (MaxPreps); Tri-State PGA junior boys 11-14 in 2024</t>
         </is>
       </c>
-      <c r="H52" s="8" t="inlineStr">
+      <c r="I52" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2278,15 +2495,20 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G53" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H53" s="8" t="inlineStr"/>
+      <c r="I53" s="8" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -2314,15 +2536,20 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G54" s="8" t="inlineStr">
+      <c r="H54" s="8" t="inlineStr">
         <is>
           <t>Probably Jimmy Brahm, PGA, former Fox Chapel assistant pro: Slippery Rock graduate who entered the golf business in 2000; identity and year both uncertain</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
+      <c r="I54" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2354,15 +2581,20 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G55" s="8" t="inlineStr">
+      <c r="H55" s="8" t="inlineStr">
         <is>
           <t>SMU sophomore in spring 2025</t>
         </is>
       </c>
-      <c r="H55" s="8" t="inlineStr">
+      <c r="I55" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2392,17 +2624,22 @@
       <c r="E56" s="7" t="n">
         <v>1981</v>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Please confirm</t>
         </is>
       </c>
-      <c r="G56" s="8" t="inlineStr">
+      <c r="H56" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025 shows 1981-07-06, identical to Eric Hellberg; one of the two is probably a copy error, so both are approximate until Fox Chapel confirms</t>
         </is>
       </c>
-      <c r="H56" s="8" t="inlineStr">
+      <c r="I56" s="8" t="inlineStr">
         <is>
           <t>The roster gives this player the same full date as another player – please check which is right</t>
         </is>
@@ -2426,13 +2663,14 @@
       </c>
       <c r="D57" s="6" t="inlineStr"/>
       <c r="E57" s="7" t="n"/>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G57" s="8" t="inlineStr"/>
-      <c r="H57" s="8" t="inlineStr">
+      <c r="H57" s="8" t="inlineStr"/>
+      <c r="I57" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2464,15 +2702,20 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G58" s="8" t="inlineStr">
+      <c r="H58" s="8" t="inlineStr">
         <is>
           <t>Shady Side Academy and GWU graduate, first job 2007; uncertain</t>
         </is>
       </c>
-      <c r="H58" s="8" t="inlineStr">
+      <c r="I58" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2504,15 +2747,20 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G59" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H59" s="8" t="inlineStr"/>
+      <c r="I59" s="8" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -2540,15 +2788,20 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G60" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H60" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr"/>
+      <c r="I60" s="8" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -2576,15 +2829,20 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G61" s="8" t="inlineStr">
+      <c r="H61" s="8" t="inlineStr">
         <is>
           <t>Age 45 in Poets &amp; Quants profile, 2025</t>
         </is>
       </c>
-      <c r="H61" s="8" t="inlineStr">
+      <c r="I61" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2608,13 +2866,14 @@
       </c>
       <c r="D62" s="6" t="inlineStr"/>
       <c r="E62" s="7" t="n"/>
-      <c r="F62" s="5" t="inlineStr">
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G62" s="8" t="inlineStr"/>
-      <c r="H62" s="8" t="inlineStr">
+      <c r="H62" s="8" t="inlineStr"/>
+      <c r="I62" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2638,13 +2897,14 @@
       </c>
       <c r="D63" s="6" t="inlineStr"/>
       <c r="E63" s="7" t="n"/>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G63" s="8" t="inlineStr"/>
-      <c r="H63" s="8" t="inlineStr">
+      <c r="H63" s="8" t="inlineStr"/>
+      <c r="I63" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2676,15 +2936,20 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G64" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H64" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H64" s="8" t="inlineStr"/>
+      <c r="I64" s="8" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -2712,15 +2977,20 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G65" s="8" t="inlineStr">
+      <c r="H65" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster: 49 in Oct 2023</t>
         </is>
       </c>
-      <c r="H65" s="8" t="inlineStr">
+      <c r="I65" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -2752,15 +3022,20 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G66" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H66" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H66" s="8" t="inlineStr"/>
+      <c r="I66" s="8" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -2788,15 +3063,20 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G67" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H67" s="8" t="inlineStr"/>
+      <c r="I67" s="8" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -2822,17 +3102,22 @@
       <c r="E68" s="7" t="n">
         <v>1972</v>
       </c>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Please confirm</t>
         </is>
       </c>
-      <c r="G68" s="8" t="inlineStr">
+      <c r="H68" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025 shows 1972-12-15, identical to Tom Delaney (Oakmont) and probably pasted; year kept as approximate until Fox Chapel confirms</t>
         </is>
       </c>
-      <c r="H68" s="8" t="inlineStr">
+      <c r="I68" s="8" t="inlineStr">
         <is>
           <t>The roster gives this player the same full date as another player – please check which is right</t>
         </is>
@@ -2856,13 +3141,14 @@
       </c>
       <c r="D69" s="6" t="inlineStr"/>
       <c r="E69" s="7" t="n"/>
-      <c r="F69" s="5" t="inlineStr">
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G69" s="8" t="inlineStr"/>
-      <c r="H69" s="8" t="inlineStr">
+      <c r="H69" s="8" t="inlineStr"/>
+      <c r="I69" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -2892,17 +3178,22 @@
       <c r="E70" s="7" t="n">
         <v>1981</v>
       </c>
-      <c r="F70" s="6" t="inlineStr">
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>Please confirm</t>
         </is>
       </c>
-      <c r="G70" s="8" t="inlineStr">
+      <c r="H70" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025 shows 1981-07-06, identical to Michael Carlin; one of the two is probably a copy error, so both are approximate until Fox Chapel confirms</t>
         </is>
       </c>
-      <c r="H70" s="8" t="inlineStr">
+      <c r="I70" s="8" t="inlineStr">
         <is>
           <t>The roster gives this player the same full date as another player – please check which is right</t>
         </is>
@@ -2934,15 +3225,20 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G71" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H71" s="8" t="inlineStr"/>
+      <c r="I71" s="8" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -2970,15 +3266,20 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G72" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H72" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H72" s="8" t="inlineStr"/>
+      <c r="I72" s="8" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -3006,15 +3307,20 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G73" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H73" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H73" s="8" t="inlineStr"/>
+      <c r="I73" s="8" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -3034,13 +3340,14 @@
       </c>
       <c r="D74" s="6" t="inlineStr"/>
       <c r="E74" s="7" t="n"/>
-      <c r="F74" s="5" t="inlineStr">
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G74" s="8" t="inlineStr"/>
-      <c r="H74" s="8" t="inlineStr">
+      <c r="H74" s="8" t="inlineStr"/>
+      <c r="I74" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3072,15 +3379,20 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G75" s="8" t="inlineStr">
+      <c r="H75" s="8" t="inlineStr">
         <is>
           <t>Shady Side Academy junior in fall 2019; WPIAL 3A runner-up 2020</t>
         </is>
       </c>
-      <c r="H75" s="8" t="inlineStr">
+      <c r="I75" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -3112,15 +3424,20 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G76" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H76" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H76" s="8" t="inlineStr"/>
+      <c r="I76" s="8" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -3148,15 +3465,20 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G77" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H77" s="8" t="inlineStr"/>
+      <c r="I77" s="8" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -3184,15 +3506,20 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G78" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H78" s="8" t="inlineStr"/>
+      <c r="I78" s="8" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -3212,13 +3539,14 @@
       </c>
       <c r="D79" s="6" t="inlineStr"/>
       <c r="E79" s="7" t="n"/>
-      <c r="F79" s="5" t="inlineStr">
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G79" s="8" t="inlineStr"/>
-      <c r="H79" s="8" t="inlineStr">
+      <c r="H79" s="8" t="inlineStr"/>
+      <c r="I79" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3242,13 +3570,14 @@
       </c>
       <c r="D80" s="6" t="inlineStr"/>
       <c r="E80" s="7" t="n"/>
-      <c r="F80" s="5" t="inlineStr">
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G80" s="8" t="inlineStr"/>
-      <c r="H80" s="8" t="inlineStr">
+      <c r="H80" s="8" t="inlineStr"/>
+      <c r="I80" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3280,15 +3609,20 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G81" s="8" t="inlineStr">
+      <c r="H81" s="8" t="inlineStr">
         <is>
           <t>Peters Township class of 2012; Saint Francis golf 2012-16</t>
         </is>
       </c>
-      <c r="H81" s="8" t="inlineStr">
+      <c r="I81" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -3312,13 +3646,14 @@
       </c>
       <c r="D82" s="6" t="inlineStr"/>
       <c r="E82" s="7" t="n"/>
-      <c r="F82" s="5" t="inlineStr">
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G82" s="8" t="inlineStr"/>
-      <c r="H82" s="8" t="inlineStr">
+      <c r="H82" s="8" t="inlineStr"/>
+      <c r="I82" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3350,15 +3685,20 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G83" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
         <is>
           <t>Georgetown men's golf roster</t>
         </is>
       </c>
-      <c r="H83" s="8" t="inlineStr"/>
+      <c r="I83" s="8" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -3386,15 +3726,20 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G84" s="8" t="inlineStr">
+      <c r="H84" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster: 60 in Oct 2023</t>
         </is>
       </c>
-      <c r="H84" s="8" t="inlineStr">
+      <c r="I84" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -3418,13 +3763,14 @@
       </c>
       <c r="D85" s="6" t="inlineStr"/>
       <c r="E85" s="7" t="n"/>
-      <c r="F85" s="5" t="inlineStr">
+      <c r="F85" s="5" t="inlineStr"/>
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G85" s="8" t="inlineStr"/>
-      <c r="H85" s="8" t="inlineStr">
+      <c r="H85" s="8" t="inlineStr"/>
+      <c r="I85" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3448,13 +3794,14 @@
       </c>
       <c r="D86" s="6" t="inlineStr"/>
       <c r="E86" s="7" t="n"/>
-      <c r="F86" s="5" t="inlineStr">
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G86" s="8" t="inlineStr"/>
-      <c r="H86" s="8" t="inlineStr">
+      <c r="H86" s="8" t="inlineStr"/>
+      <c r="I86" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3486,15 +3833,20 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G87" s="8" t="inlineStr">
+      <c r="H87" s="8" t="inlineStr">
         <is>
           <t>Gus Schroeder Jr., Schroeder Industries president since 2005; rough estimate, father (also Gus, b. c. 1940) died c. 2000</t>
         </is>
       </c>
-      <c r="H87" s="8" t="inlineStr">
+      <c r="I87" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -3518,13 +3870,14 @@
       </c>
       <c r="D88" s="6" t="inlineStr"/>
       <c r="E88" s="7" t="n"/>
-      <c r="F88" s="5" t="inlineStr">
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G88" s="8" t="inlineStr"/>
-      <c r="H88" s="8" t="inlineStr">
+      <c r="H88" s="8" t="inlineStr"/>
+      <c r="I88" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3556,15 +3909,20 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G89" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H89" s="8" t="inlineStr"/>
+      <c r="I89" s="8" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -3584,13 +3942,14 @@
       </c>
       <c r="D90" s="6" t="inlineStr"/>
       <c r="E90" s="7" t="n"/>
-      <c r="F90" s="5" t="inlineStr">
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G90" s="8" t="inlineStr"/>
-      <c r="H90" s="8" t="inlineStr">
+      <c r="H90" s="8" t="inlineStr"/>
+      <c r="I90" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3622,15 +3981,20 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G91" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H91" s="8" t="inlineStr"/>
+      <c r="I91" s="8" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -3658,15 +4022,20 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G92" s="8" t="inlineStr">
+      <c r="H92" s="8" t="inlineStr">
         <is>
           <t>Peters Township HS golf 2010 alongside Tommy Nettles; uncertain, same name only</t>
         </is>
       </c>
-      <c r="H92" s="8" t="inlineStr">
+      <c r="I92" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -3690,13 +4059,14 @@
       </c>
       <c r="D93" s="6" t="inlineStr"/>
       <c r="E93" s="7" t="n"/>
-      <c r="F93" s="5" t="inlineStr">
+      <c r="F93" s="5" t="inlineStr"/>
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G93" s="8" t="inlineStr"/>
-      <c r="H93" s="8" t="inlineStr">
+      <c r="H93" s="8" t="inlineStr"/>
+      <c r="I93" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3720,13 +4090,14 @@
       </c>
       <c r="D94" s="6" t="inlineStr"/>
       <c r="E94" s="7" t="n"/>
-      <c r="F94" s="5" t="inlineStr">
+      <c r="F94" s="5" t="inlineStr"/>
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G94" s="8" t="inlineStr"/>
-      <c r="H94" s="8" t="inlineStr">
+      <c r="H94" s="8" t="inlineStr"/>
+      <c r="I94" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3750,13 +4121,14 @@
       </c>
       <c r="D95" s="6" t="inlineStr"/>
       <c r="E95" s="7" t="n"/>
-      <c r="F95" s="5" t="inlineStr">
+      <c r="F95" s="5" t="inlineStr"/>
+      <c r="G95" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G95" s="8" t="inlineStr"/>
-      <c r="H95" s="8" t="inlineStr">
+      <c r="H95" s="8" t="inlineStr"/>
+      <c r="I95" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3780,13 +4152,14 @@
       </c>
       <c r="D96" s="6" t="inlineStr"/>
       <c r="E96" s="7" t="n"/>
-      <c r="F96" s="5" t="inlineStr">
+      <c r="F96" s="5" t="inlineStr"/>
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G96" s="8" t="inlineStr"/>
-      <c r="H96" s="8" t="inlineStr">
+      <c r="H96" s="8" t="inlineStr"/>
+      <c r="I96" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3810,13 +4183,14 @@
       </c>
       <c r="D97" s="6" t="inlineStr"/>
       <c r="E97" s="7" t="n"/>
-      <c r="F97" s="5" t="inlineStr">
+      <c r="F97" s="5" t="inlineStr"/>
+      <c r="G97" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G97" s="8" t="inlineStr"/>
-      <c r="H97" s="8" t="inlineStr">
+      <c r="H97" s="8" t="inlineStr"/>
+      <c r="I97" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3848,15 +4222,20 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G98" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H98" s="8" t="inlineStr"/>
+      <c r="I98" s="8" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -3884,15 +4263,20 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G99" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H99" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H99" s="8" t="inlineStr"/>
+      <c r="I99" s="8" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -3920,15 +4304,20 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G100" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H100" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H100" s="8" t="inlineStr"/>
+      <c r="I100" s="8" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
@@ -3948,13 +4337,14 @@
       </c>
       <c r="D101" s="6" t="inlineStr"/>
       <c r="E101" s="7" t="n"/>
-      <c r="F101" s="5" t="inlineStr">
+      <c r="F101" s="5" t="inlineStr"/>
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G101" s="8" t="inlineStr"/>
-      <c r="H101" s="8" t="inlineStr">
+      <c r="H101" s="8" t="inlineStr"/>
+      <c r="I101" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -3986,15 +4376,20 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G102" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H102" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H102" s="8" t="inlineStr"/>
+      <c r="I102" s="8" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
@@ -4022,15 +4417,20 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G103" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H103" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H103" s="8" t="inlineStr"/>
+      <c r="I103" s="8" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -4058,15 +4458,20 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G104" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H104" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H104" s="8" t="inlineStr"/>
+      <c r="I104" s="8" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -4094,15 +4499,20 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G105" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G105" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H105" s="8" t="inlineStr"/>
+      <c r="I105" s="8" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -4130,15 +4540,20 @@
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G106" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H106" s="8" t="inlineStr"/>
+      <c r="I106" s="8" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -4166,15 +4581,20 @@
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G107" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H107" s="8" t="inlineStr"/>
+      <c r="I107" s="8" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -4202,15 +4622,20 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G108" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H108" s="8" t="inlineStr"/>
+      <c r="I108" s="8" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -4238,15 +4663,20 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G109" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G109" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H109" s="8" t="inlineStr"/>
+      <c r="I109" s="8" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -4274,15 +4704,20 @@
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G110" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H110" s="8" t="inlineStr"/>
+      <c r="I110" s="8" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -4310,15 +4745,20 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G111" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G111" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025; the roster's own age column (50 in Oct 2023) agrees. Clint Guyaux (Fox Chapel) carries the same date, probably pasted from this row</t>
         </is>
       </c>
-      <c r="H111" s="8" t="inlineStr"/>
+      <c r="I111" s="8" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -4346,15 +4786,20 @@
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G112" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H112" s="8" t="inlineStr"/>
+      <c r="I112" s="8" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
@@ -4382,15 +4827,20 @@
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G113" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H113" s="8" t="inlineStr"/>
+      <c r="I113" s="8" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -4418,15 +4868,20 @@
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G114" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H114" s="8" t="inlineStr"/>
+      <c r="I114" s="8" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
@@ -4446,13 +4901,14 @@
       </c>
       <c r="D115" s="6" t="inlineStr"/>
       <c r="E115" s="7" t="n"/>
-      <c r="F115" s="5" t="inlineStr">
+      <c r="F115" s="5" t="inlineStr"/>
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G115" s="8" t="inlineStr"/>
-      <c r="H115" s="8" t="inlineStr">
+      <c r="H115" s="8" t="inlineStr"/>
+      <c r="I115" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -4484,15 +4940,20 @@
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G116" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H116" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H116" s="8" t="inlineStr"/>
+      <c r="I116" s="8" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
@@ -4520,15 +4981,20 @@
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G117" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H117" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H117" s="8" t="inlineStr"/>
+      <c r="I117" s="8" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -4556,15 +5022,20 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G118" s="8" t="inlineStr">
+      <c r="H118" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster: 28 in Oct 2023; Emory golf 2014-18 agrees</t>
         </is>
       </c>
-      <c r="H118" s="8" t="inlineStr">
+      <c r="I118" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -4596,15 +5067,20 @@
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G119" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G119" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H119" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H119" s="8" t="inlineStr"/>
+      <c r="I119" s="8" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -4632,15 +5108,20 @@
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G120" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G120" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H120" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H120" s="8" t="inlineStr"/>
+      <c r="I120" s="8" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
@@ -4668,15 +5149,20 @@
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G121" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G121" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H121" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H121" s="8" t="inlineStr"/>
+      <c r="I121" s="8" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -4704,15 +5190,20 @@
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G122" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G122" s="8" t="inlineStr">
+      <c r="H122" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster: 30 in Oct 2023</t>
         </is>
       </c>
-      <c r="H122" s="8" t="inlineStr">
+      <c r="I122" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -4744,15 +5235,20 @@
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G123" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H123" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H123" s="8" t="inlineStr"/>
+      <c r="I123" s="8" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -4780,15 +5276,20 @@
       </c>
       <c r="F124" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G124" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G124" s="8" t="inlineStr">
+      <c r="H124" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster: 20 in Oct 2023</t>
         </is>
       </c>
-      <c r="H124" s="8" t="inlineStr">
+      <c r="I124" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -4820,15 +5321,20 @@
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G125" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G125" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H125" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H125" s="8" t="inlineStr"/>
+      <c r="I125" s="8" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -4856,15 +5362,20 @@
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G126" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H126" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H126" s="8" t="inlineStr"/>
+      <c r="I126" s="8" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
@@ -4892,15 +5403,20 @@
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G127" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G127" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H127" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H127" s="8" t="inlineStr"/>
+      <c r="I127" s="8" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -4928,15 +5444,20 @@
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G128" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G128" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H128" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H128" s="8" t="inlineStr"/>
+      <c r="I128" s="8" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -4964,15 +5485,20 @@
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G129" s="8" t="inlineStr">
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G129" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H129" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H129" s="8" t="inlineStr"/>
+      <c r="I129" s="8" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -5000,15 +5526,20 @@
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G130" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H130" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H130" s="8" t="inlineStr"/>
+      <c r="I130" s="8" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
@@ -5036,15 +5567,20 @@
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G131" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H131" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H131" s="8" t="inlineStr"/>
+      <c r="I131" s="8" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -5072,15 +5608,20 @@
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G132" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G132" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H132" s="8" t="inlineStr">
         <is>
           <t>PGA Tour player bio (Tom Nettles, McMurray PA)</t>
         </is>
       </c>
-      <c r="H132" s="8" t="inlineStr"/>
+      <c r="I132" s="8" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
@@ -5108,15 +5649,20 @@
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G133" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H133" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H133" s="8" t="inlineStr"/>
+      <c r="I133" s="8" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -5144,15 +5690,20 @@
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G134" s="8" t="inlineStr">
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G134" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H134" s="8" t="inlineStr">
         <is>
           <t>High Point University men's golf roster</t>
         </is>
       </c>
-      <c r="H134" s="8" t="inlineStr"/>
+      <c r="I134" s="8" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -5180,15 +5731,20 @@
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G135" s="8" t="inlineStr">
+      <c r="H135" s="8" t="inlineStr">
         <is>
           <t>Central Catholic class of 2023, Notre Dame class of 2027; 18 on the Oakmont roster in Oct 2023</t>
         </is>
       </c>
-      <c r="H135" s="8" t="inlineStr">
+      <c r="I135" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5220,15 +5776,20 @@
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G136" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G136" s="8" t="inlineStr">
+      <c r="H136" s="8" t="inlineStr">
         <is>
           <t>Franklin Regional class of 2023; signed with Youngstown State for 2023-24</t>
         </is>
       </c>
-      <c r="H136" s="8" t="inlineStr">
+      <c r="I136" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5260,15 +5821,20 @@
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G137" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H137" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H137" s="8" t="inlineStr"/>
+      <c r="I137" s="8" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -5296,15 +5862,20 @@
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G138" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G138" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H138" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H138" s="8" t="inlineStr"/>
+      <c r="I138" s="8" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
@@ -5332,15 +5903,20 @@
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G139" s="8" t="inlineStr">
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H139" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H139" s="8" t="inlineStr"/>
+      <c r="I139" s="8" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -5368,15 +5944,20 @@
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G140" s="8" t="inlineStr">
+      <c r="H140" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster: 56 in Oct 2023</t>
         </is>
       </c>
-      <c r="H140" s="8" t="inlineStr">
+      <c r="I140" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5408,15 +5989,20 @@
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G141" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H141" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H141" s="8" t="inlineStr"/>
+      <c r="I141" s="8" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -5444,15 +6030,20 @@
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G142" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H142" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H142" s="8" t="inlineStr"/>
+      <c r="I142" s="8" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
@@ -5480,15 +6071,20 @@
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G143" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H143" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H143" s="8" t="inlineStr"/>
+      <c r="I143" s="8" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -5516,15 +6112,20 @@
       </c>
       <c r="F144" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G144" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H144" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H144" s="8" t="inlineStr"/>
+      <c r="I144" s="8" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
@@ -5552,15 +6153,20 @@
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G145" s="8" t="inlineStr">
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H145" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H145" s="8" t="inlineStr"/>
+      <c r="I145" s="8" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -5588,15 +6194,20 @@
       </c>
       <c r="F146" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G146" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G146" s="8" t="inlineStr">
+      <c r="H146" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster: 30 in Oct 2023</t>
         </is>
       </c>
-      <c r="H146" s="8" t="inlineStr">
+      <c r="I146" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5628,15 +6239,20 @@
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="G147" s="8" t="inlineStr">
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="H147" s="8" t="inlineStr">
         <is>
           <t>Oakmont age roster, Aug 2025</t>
         </is>
       </c>
-      <c r="H147" s="8" t="inlineStr"/>
+      <c r="I147" s="8" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -5656,13 +6272,14 @@
       </c>
       <c r="D148" s="6" t="inlineStr"/>
       <c r="E148" s="7" t="n"/>
-      <c r="F148" s="5" t="inlineStr">
+      <c r="F148" s="5" t="inlineStr"/>
+      <c r="G148" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G148" s="8" t="inlineStr"/>
-      <c r="H148" s="8" t="inlineStr">
+      <c r="H148" s="8" t="inlineStr"/>
+      <c r="I148" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5686,13 +6303,14 @@
       </c>
       <c r="D149" s="6" t="inlineStr"/>
       <c r="E149" s="7" t="n"/>
-      <c r="F149" s="5" t="inlineStr">
+      <c r="F149" s="5" t="inlineStr"/>
+      <c r="G149" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G149" s="8" t="inlineStr"/>
-      <c r="H149" s="8" t="inlineStr">
+      <c r="H149" s="8" t="inlineStr"/>
+      <c r="I149" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5724,15 +6342,20 @@
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G150" s="8" t="inlineStr">
+      <c r="H150" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel HS freshman in 2007, then prep school, class of 2011/12 (Tommy Leech); Hartford golf senior 2015-16</t>
         </is>
       </c>
-      <c r="H150" s="8" t="inlineStr">
+      <c r="I150" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5756,13 +6379,14 @@
       </c>
       <c r="D151" s="6" t="inlineStr"/>
       <c r="E151" s="7" t="n"/>
-      <c r="F151" s="5" t="inlineStr">
+      <c r="F151" s="5" t="inlineStr"/>
+      <c r="G151" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G151" s="8" t="inlineStr"/>
-      <c r="H151" s="8" t="inlineStr">
+      <c r="H151" s="8" t="inlineStr"/>
+      <c r="I151" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5786,13 +6410,14 @@
       </c>
       <c r="D152" s="6" t="inlineStr"/>
       <c r="E152" s="7" t="n"/>
-      <c r="F152" s="5" t="inlineStr">
+      <c r="F152" s="5" t="inlineStr"/>
+      <c r="G152" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G152" s="8" t="inlineStr"/>
-      <c r="H152" s="8" t="inlineStr">
+      <c r="H152" s="8" t="inlineStr"/>
+      <c r="I152" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5818,13 +6443,22 @@
       <c r="E153" s="7" t="n"/>
       <c r="F153" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G153" s="8" t="inlineStr"/>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>Band only</t>
+        </is>
+      </c>
       <c r="H153" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Tommy Leech, Oct 2026</t>
+        </is>
+      </c>
+      <c r="I153" s="8" t="inlineStr">
+        <is>
+          <t>Only an age band is known – a year would be better</t>
         </is>
       </c>
     </row>
@@ -5846,13 +6480,14 @@
       </c>
       <c r="D154" s="6" t="inlineStr"/>
       <c r="E154" s="7" t="n"/>
-      <c r="F154" s="5" t="inlineStr">
+      <c r="F154" s="5" t="inlineStr"/>
+      <c r="G154" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G154" s="8" t="inlineStr"/>
-      <c r="H154" s="8" t="inlineStr">
+      <c r="H154" s="8" t="inlineStr"/>
+      <c r="I154" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5884,15 +6519,20 @@
       </c>
       <c r="F155" s="5" t="inlineStr">
         <is>
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G155" s="8" t="inlineStr">
+      <c r="H155" s="8" t="inlineStr">
         <is>
           <t>Pittsburgh entrant in 2014 U.S. Junior Amateur qualifying (under 19); uncertain by a year or two</t>
         </is>
       </c>
-      <c r="H155" s="8" t="inlineStr">
+      <c r="I155" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -5916,13 +6556,14 @@
       </c>
       <c r="D156" s="6" t="inlineStr"/>
       <c r="E156" s="7" t="n"/>
-      <c r="F156" s="5" t="inlineStr">
+      <c r="F156" s="5" t="inlineStr"/>
+      <c r="G156" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G156" s="8" t="inlineStr"/>
-      <c r="H156" s="8" t="inlineStr">
+      <c r="H156" s="8" t="inlineStr"/>
+      <c r="I156" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -5948,13 +6589,22 @@
       <c r="E157" s="7" t="n"/>
       <c r="F157" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G157" s="8" t="inlineStr"/>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>Band only</t>
+        </is>
+      </c>
       <c r="H157" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Tommy Leech, Oct 2026</t>
+        </is>
+      </c>
+      <c r="I157" s="8" t="inlineStr">
+        <is>
+          <t>Only an age band is known – a year would be better</t>
         </is>
       </c>
     </row>
@@ -5976,13 +6626,14 @@
       </c>
       <c r="D158" s="6" t="inlineStr"/>
       <c r="E158" s="7" t="n"/>
-      <c r="F158" s="5" t="inlineStr">
+      <c r="F158" s="5" t="inlineStr"/>
+      <c r="G158" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G158" s="8" t="inlineStr"/>
-      <c r="H158" s="8" t="inlineStr">
+      <c r="H158" s="8" t="inlineStr"/>
+      <c r="I158" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6014,15 +6665,20 @@
       </c>
       <c r="F159" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G159" s="8" t="inlineStr">
+      <c r="H159" s="8" t="inlineStr">
         <is>
           <t>Age 45 in Poets &amp; Quants profile, 2025</t>
         </is>
       </c>
-      <c r="H159" s="8" t="inlineStr">
+      <c r="I159" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6046,13 +6702,14 @@
       </c>
       <c r="D160" s="6" t="inlineStr"/>
       <c r="E160" s="7" t="n"/>
-      <c r="F160" s="5" t="inlineStr">
+      <c r="F160" s="5" t="inlineStr"/>
+      <c r="G160" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G160" s="8" t="inlineStr"/>
-      <c r="H160" s="8" t="inlineStr">
+      <c r="H160" s="8" t="inlineStr"/>
+      <c r="I160" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6076,13 +6733,14 @@
       </c>
       <c r="D161" s="6" t="inlineStr"/>
       <c r="E161" s="7" t="n"/>
-      <c r="F161" s="5" t="inlineStr">
+      <c r="F161" s="5" t="inlineStr"/>
+      <c r="G161" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G161" s="8" t="inlineStr"/>
-      <c r="H161" s="8" t="inlineStr">
+      <c r="H161" s="8" t="inlineStr"/>
+      <c r="I161" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6106,13 +6764,14 @@
       </c>
       <c r="D162" s="6" t="inlineStr"/>
       <c r="E162" s="7" t="n"/>
-      <c r="F162" s="5" t="inlineStr">
+      <c r="F162" s="5" t="inlineStr"/>
+      <c r="G162" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G162" s="8" t="inlineStr"/>
-      <c r="H162" s="8" t="inlineStr">
+      <c r="H162" s="8" t="inlineStr"/>
+      <c r="I162" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6136,13 +6795,14 @@
       </c>
       <c r="D163" s="6" t="inlineStr"/>
       <c r="E163" s="7" t="n"/>
-      <c r="F163" s="5" t="inlineStr">
+      <c r="F163" s="5" t="inlineStr"/>
+      <c r="G163" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G163" s="8" t="inlineStr"/>
-      <c r="H163" s="8" t="inlineStr">
+      <c r="H163" s="8" t="inlineStr"/>
+      <c r="I163" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6166,13 +6826,14 @@
       </c>
       <c r="D164" s="6" t="inlineStr"/>
       <c r="E164" s="7" t="n"/>
-      <c r="F164" s="5" t="inlineStr">
+      <c r="F164" s="5" t="inlineStr"/>
+      <c r="G164" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G164" s="8" t="inlineStr"/>
-      <c r="H164" s="8" t="inlineStr">
+      <c r="H164" s="8" t="inlineStr"/>
+      <c r="I164" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6196,13 +6857,14 @@
       </c>
       <c r="D165" s="6" t="inlineStr"/>
       <c r="E165" s="7" t="n"/>
-      <c r="F165" s="5" t="inlineStr">
+      <c r="F165" s="5" t="inlineStr"/>
+      <c r="G165" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G165" s="8" t="inlineStr"/>
-      <c r="H165" s="8" t="inlineStr">
+      <c r="H165" s="8" t="inlineStr"/>
+      <c r="I165" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6234,15 +6896,20 @@
       </c>
       <c r="F166" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G166" s="8" t="inlineStr">
+      <c r="H166" s="8" t="inlineStr">
         <is>
           <t>Shady Side Academy; senior on the South Carolina golf roster 2015-16</t>
         </is>
       </c>
-      <c r="H166" s="8" t="inlineStr">
+      <c r="I166" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6274,15 +6941,20 @@
       </c>
       <c r="F167" s="5" t="inlineStr">
         <is>
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G167" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G167" s="8" t="inlineStr">
+      <c r="H167" s="8" t="inlineStr">
         <is>
           <t>Shaler graduate; Findlay golf, senior in 2023; uncertain by a year or two</t>
         </is>
       </c>
-      <c r="H167" s="8" t="inlineStr">
+      <c r="I167" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6304,17 +6976,32 @@
           <t>2012–2023</t>
         </is>
       </c>
-      <c r="D168" s="6" t="inlineStr"/>
-      <c r="E168" s="7" t="n"/>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+      <c r="E168" s="7" t="n">
+        <v>1984</v>
+      </c>
       <c r="F168" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G168" s="8" t="inlineStr"/>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>Approximate</t>
+        </is>
+      </c>
       <c r="H168" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>About 42 in Oct 2026 (Tommy Leech)</t>
+        </is>
+      </c>
+      <c r="I168" s="8" t="inlineStr">
+        <is>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6334,17 +7021,32 @@
           <t>2015–2025</t>
         </is>
       </c>
-      <c r="D169" s="6" t="inlineStr"/>
-      <c r="E169" s="7" t="n"/>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="E169" s="7" t="n">
+        <v>1990</v>
+      </c>
       <c r="F169" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G169" s="8" t="inlineStr"/>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G169" s="5" t="inlineStr">
+        <is>
+          <t>Approximate</t>
+        </is>
+      </c>
       <c r="H169" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>About 36 in Oct 2026 (Tommy Leech)</t>
+        </is>
+      </c>
+      <c r="I169" s="8" t="inlineStr">
+        <is>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -6374,15 +7076,20 @@
       </c>
       <c r="F170" s="5" t="inlineStr">
         <is>
+          <t>30–39</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G170" s="8" t="inlineStr">
+      <c r="H170" s="8" t="inlineStr">
         <is>
           <t>Deer Lakes; Penn State Behrend golf 2009-11</t>
         </is>
       </c>
-      <c r="H170" s="8" t="inlineStr">
+      <c r="I170" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6406,13 +7113,14 @@
       </c>
       <c r="D171" s="6" t="inlineStr"/>
       <c r="E171" s="7" t="n"/>
-      <c r="F171" s="5" t="inlineStr">
+      <c r="F171" s="5" t="inlineStr"/>
+      <c r="G171" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G171" s="8" t="inlineStr"/>
-      <c r="H171" s="8" t="inlineStr">
+      <c r="H171" s="8" t="inlineStr"/>
+      <c r="I171" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6436,13 +7144,14 @@
       </c>
       <c r="D172" s="6" t="inlineStr"/>
       <c r="E172" s="7" t="n"/>
-      <c r="F172" s="5" t="inlineStr">
+      <c r="F172" s="5" t="inlineStr"/>
+      <c r="G172" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G172" s="8" t="inlineStr"/>
-      <c r="H172" s="8" t="inlineStr">
+      <c r="H172" s="8" t="inlineStr"/>
+      <c r="I172" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6468,13 +7177,22 @@
       <c r="E173" s="7" t="n"/>
       <c r="F173" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G173" s="8" t="inlineStr"/>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="G173" s="5" t="inlineStr">
+        <is>
+          <t>Band only</t>
+        </is>
+      </c>
       <c r="H173" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Tommy Leech, Oct 2026</t>
+        </is>
+      </c>
+      <c r="I173" s="8" t="inlineStr">
+        <is>
+          <t>Only an age band is known – a year would be better</t>
         </is>
       </c>
     </row>
@@ -6504,15 +7222,20 @@
       </c>
       <c r="F174" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G174" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G174" s="8" t="inlineStr">
+      <c r="H174" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel HS junior in fall 2019 (WPIAL 3A, T3)</t>
         </is>
       </c>
-      <c r="H174" s="8" t="inlineStr">
+      <c r="I174" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6536,13 +7259,14 @@
       </c>
       <c r="D175" s="6" t="inlineStr"/>
       <c r="E175" s="7" t="n"/>
-      <c r="F175" s="5" t="inlineStr">
+      <c r="F175" s="5" t="inlineStr"/>
+      <c r="G175" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G175" s="8" t="inlineStr"/>
-      <c r="H175" s="8" t="inlineStr">
+      <c r="H175" s="8" t="inlineStr"/>
+      <c r="I175" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6574,15 +7298,20 @@
       </c>
       <c r="F176" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G176" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G176" s="8" t="inlineStr">
+      <c r="H176" s="8" t="inlineStr">
         <is>
           <t>Serra Catholic; senior on the Marshall golf roster 2007-08</t>
         </is>
       </c>
-      <c r="H176" s="8" t="inlineStr">
+      <c r="I176" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6614,15 +7343,20 @@
       </c>
       <c r="F177" s="5" t="inlineStr">
         <is>
+          <t>40–49</t>
+        </is>
+      </c>
+      <c r="G177" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G177" s="8" t="inlineStr">
+      <c r="H177" s="8" t="inlineStr">
         <is>
           <t>Allegheny College class of 2005 (athletics hall of fame)</t>
         </is>
       </c>
-      <c r="H177" s="8" t="inlineStr">
+      <c r="I177" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6646,13 +7380,14 @@
       </c>
       <c r="D178" s="6" t="inlineStr"/>
       <c r="E178" s="7" t="n"/>
-      <c r="F178" s="5" t="inlineStr">
+      <c r="F178" s="5" t="inlineStr"/>
+      <c r="G178" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G178" s="8" t="inlineStr"/>
-      <c r="H178" s="8" t="inlineStr">
+      <c r="H178" s="8" t="inlineStr"/>
+      <c r="I178" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6676,13 +7411,14 @@
       </c>
       <c r="D179" s="6" t="inlineStr"/>
       <c r="E179" s="7" t="n"/>
-      <c r="F179" s="5" t="inlineStr">
+      <c r="F179" s="5" t="inlineStr"/>
+      <c r="G179" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G179" s="8" t="inlineStr"/>
-      <c r="H179" s="8" t="inlineStr">
+      <c r="H179" s="8" t="inlineStr"/>
+      <c r="I179" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6714,15 +7450,20 @@
       </c>
       <c r="F180" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G180" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G180" s="8" t="inlineStr">
+      <c r="H180" s="8" t="inlineStr">
         <is>
           <t>Shady Side Academy sophomore in fall 2018 (IPSL medalist)</t>
         </is>
       </c>
-      <c r="H180" s="8" t="inlineStr">
+      <c r="I180" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6746,13 +7487,14 @@
       </c>
       <c r="D181" s="6" t="inlineStr"/>
       <c r="E181" s="7" t="n"/>
-      <c r="F181" s="5" t="inlineStr">
+      <c r="F181" s="5" t="inlineStr"/>
+      <c r="G181" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G181" s="8" t="inlineStr"/>
-      <c r="H181" s="8" t="inlineStr">
+      <c r="H181" s="8" t="inlineStr"/>
+      <c r="I181" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6776,13 +7518,14 @@
       </c>
       <c r="D182" s="6" t="inlineStr"/>
       <c r="E182" s="7" t="n"/>
-      <c r="F182" s="5" t="inlineStr">
+      <c r="F182" s="5" t="inlineStr"/>
+      <c r="G182" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G182" s="8" t="inlineStr"/>
-      <c r="H182" s="8" t="inlineStr">
+      <c r="H182" s="8" t="inlineStr"/>
+      <c r="I182" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6806,13 +7549,14 @@
       </c>
       <c r="D183" s="6" t="inlineStr"/>
       <c r="E183" s="7" t="n"/>
-      <c r="F183" s="5" t="inlineStr">
+      <c r="F183" s="5" t="inlineStr"/>
+      <c r="G183" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G183" s="8" t="inlineStr"/>
-      <c r="H183" s="8" t="inlineStr">
+      <c r="H183" s="8" t="inlineStr"/>
+      <c r="I183" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6836,13 +7580,14 @@
       </c>
       <c r="D184" s="6" t="inlineStr"/>
       <c r="E184" s="7" t="n"/>
-      <c r="F184" s="5" t="inlineStr">
+      <c r="F184" s="5" t="inlineStr"/>
+      <c r="G184" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G184" s="8" t="inlineStr"/>
-      <c r="H184" s="8" t="inlineStr">
+      <c r="H184" s="8" t="inlineStr"/>
+      <c r="I184" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6866,13 +7611,14 @@
       </c>
       <c r="D185" s="6" t="inlineStr"/>
       <c r="E185" s="7" t="n"/>
-      <c r="F185" s="5" t="inlineStr">
+      <c r="F185" s="5" t="inlineStr"/>
+      <c r="G185" s="5" t="inlineStr">
         <is>
           <t>Missing</t>
         </is>
       </c>
-      <c r="G185" s="8" t="inlineStr"/>
-      <c r="H185" s="8" t="inlineStr">
+      <c r="H185" s="8" t="inlineStr"/>
+      <c r="I185" s="8" t="inlineStr">
         <is>
           <t>Please add</t>
         </is>
@@ -6904,15 +7650,20 @@
       </c>
       <c r="F186" s="5" t="inlineStr">
         <is>
+          <t>25–29</t>
+        </is>
+      </c>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G186" s="8" t="inlineStr">
+      <c r="H186" s="8" t="inlineStr">
         <is>
           <t>Pine-Richland golfer at the 2018 PIAA championship; class year not found, uncertain</t>
         </is>
       </c>
-      <c r="H186" s="8" t="inlineStr">
+      <c r="I186" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
@@ -6944,22 +7695,27 @@
       </c>
       <c r="F187" s="5" t="inlineStr">
         <is>
+          <t>Under 25</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
           <t>Approximate</t>
         </is>
       </c>
-      <c r="G187" s="8" t="inlineStr">
+      <c r="H187" s="8" t="inlineStr">
         <is>
           <t>Fox Chapel HS junior in fall 2020</t>
         </is>
       </c>
-      <c r="H187" s="8" t="inlineStr">
+      <c r="I187" s="8" t="inlineStr">
         <is>
           <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H187"/>
+  <autoFilter ref="A5:I187"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6970,7 +7726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6978,7 +7734,8 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7016,6 +7773,11 @@
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
+          <t>Band only</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
+        <is>
           <t>Missing</t>
         </is>
       </c>
@@ -7039,6 +7801,9 @@
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7061,6 +7826,9 @@
         <v>3</v>
       </c>
       <c r="F5" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="11" t="n">
         <v>22</v>
       </c>
     </row>
@@ -7083,6 +7851,9 @@
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -7099,13 +7870,16 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>28</v>
+        <v>3</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -7121,25 +7895,28 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>53</v>
+        <v>3</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Status key: Recorded = full or month date from a roster or public record. Approximate = year inferred from an age or school class. Please confirm = roster date duplicated between two players. Missing = nothing on file.</t>
+          <t>Status key: Recorded = full or month date from a roster or public record. Approximate = year inferred from an age or school class. Please confirm = roster date duplicated between two players. Band only = an age band but no year. Missing = nothing on file.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Full names for seven initials-only players; six years from college graduation
Astorino, Barker, Kelly, Rudolf, Russell, Don Smith and Fricke get the
first names the clubs' age rosters use. Birth years for all but Smith
are graduation year minus 22, from Tommy, stored as approximate.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>L. Astorino</t>
+          <t>Lou Astorino</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -2254,18 +2254,32 @@
           <t>2017</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>1975</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>1975</v>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 1997 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I46" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2291,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>W. Barker</t>
+          <t>Watson Barker</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -2285,18 +2299,32 @@
           <t>2018–2019</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr"/>
-      <c r="E47" s="7" t="n"/>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>1977</v>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>40–49</t>
+        </is>
+      </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 1999 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3379,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>T. Kelly</t>
+          <t>Trey Kelly</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3359,18 +3387,32 @@
           <t>2017</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr"/>
-      <c r="E73" s="7" t="n"/>
-      <c r="F73" s="5" t="inlineStr"/>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>1999</v>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>25–29</t>
+        </is>
+      </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H73" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H73" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2021 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3824,7 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>C. Rudolf</t>
+          <t>Chris Rudolf</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -3790,18 +3832,32 @@
           <t>2017–2021</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr"/>
-      <c r="E84" s="7" t="n"/>
-      <c r="F84" s="5" t="inlineStr"/>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="n">
+        <v>1988</v>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>30–39</t>
+        </is>
+      </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H84" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2010 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I84" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3869,7 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>R. Russell</t>
+          <t>Randy Russell</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -3821,18 +3877,32 @@
           <t>2016–2020</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr"/>
-      <c r="E85" s="7" t="n"/>
-      <c r="F85" s="5" t="inlineStr"/>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="n">
+        <v>1969</v>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H85" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 1991 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I85" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -3975,7 +4045,7 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>D. Smith</t>
+          <t>Don Smith</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -4962,7 +5032,7 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Fricke</t>
+          <t>Jackson Fricke</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
@@ -4970,18 +5040,32 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr"/>
-      <c r="E114" s="7" t="n"/>
-      <c r="F114" s="5" t="inlineStr"/>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="n">
+        <v>2003</v>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Under 25</t>
+        </is>
+      </c>
       <c r="G114" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H114" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2025 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I114" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8155,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>3</v>
@@ -8080,7 +8164,7 @@
         <v>4</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -8096,7 +8180,7 @@
         <v>40</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
@@ -8105,7 +8189,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -8146,7 +8230,7 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
@@ -8155,7 +8239,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Henry McCrady: c. 2007, high school class of 2025 (Tommy)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -3600,18 +3600,32 @@
           <t>2023–2025</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr"/>
-      <c r="E78" s="7" t="n"/>
-      <c r="F78" s="5" t="inlineStr"/>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>2007</v>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Under 25</t>
+        </is>
+      </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H78" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
+          <t>High school class of 2025 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8155,7 +8169,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>3</v>
@@ -8164,7 +8178,7 @@
         <v>4</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -8230,7 +8244,7 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
@@ -8239,7 +8253,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Phil Compeau: name and c. 1986, college class of 2008 (Tommy)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -6675,7 +6675,7 @@
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>P. Compeau</t>
+          <t>Phil Compeau</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
@@ -6683,18 +6683,32 @@
           <t>2018</t>
         </is>
       </c>
-      <c r="D153" s="6" t="inlineStr"/>
-      <c r="E153" s="7" t="n"/>
-      <c r="F153" s="5" t="inlineStr"/>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>1986</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="n">
+        <v>1986</v>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>40–49</t>
+        </is>
+      </c>
       <c r="G153" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H153" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H153" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2008 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I153" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8233,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
@@ -8228,7 +8242,7 @@
         <v>8</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -8244,7 +8258,7 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
@@ -8253,7 +8267,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Matt Fisch: c. 1996, college class of 2018 (Tommy)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -7062,18 +7062,32 @@
           <t>2014–2021</t>
         </is>
       </c>
-      <c r="D162" s="6" t="inlineStr"/>
-      <c r="E162" s="7" t="n"/>
-      <c r="F162" s="5" t="inlineStr"/>
+      <c r="D162" s="6" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="E162" s="7" t="n">
+        <v>1996</v>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>30–39</t>
+        </is>
+      </c>
       <c r="G162" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H162" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H162" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2018 (Tommy Leech); older brother of Pitt's Aidan Fisch (b. 2000)</t>
+        </is>
+      </c>
       <c r="I162" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8233,7 +8247,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
@@ -8242,7 +8256,7 @@
         <v>8</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -8258,7 +8272,7 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
@@ -8267,7 +8281,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Mike Gielarowski: c. 1988, college class of 2010 (Tommy)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -7107,18 +7107,32 @@
           <t>2021–2025</t>
         </is>
       </c>
-      <c r="D163" s="6" t="inlineStr"/>
-      <c r="E163" s="7" t="n"/>
-      <c r="F163" s="5" t="inlineStr"/>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="E163" s="7" t="n">
+        <v>1988</v>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>30–39</t>
+        </is>
+      </c>
       <c r="G163" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H163" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H163" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2010 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I163" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8247,7 +8261,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
@@ -8256,7 +8270,7 @@
         <v>8</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -8272,7 +8286,7 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
@@ -8281,7 +8295,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Ben Sera (name, c. 1988) and David Koi (60+ band), from Tommy
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/diebold-birth-dates.xlsx
+++ b/reports/diebold-birth-dates.xlsx
@@ -7424,16 +7424,24 @@
       </c>
       <c r="D170" s="6" t="inlineStr"/>
       <c r="E170" s="7" t="n"/>
-      <c r="F170" s="5" t="inlineStr"/>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
       <c r="G170" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H170" s="8" t="inlineStr"/>
+          <t>Band only</t>
+        </is>
+      </c>
+      <c r="H170" s="8" t="inlineStr">
+        <is>
+          <t>60+ per Tommy Leech, Oct 2026 (bands stop at 50+)</t>
+        </is>
+      </c>
       <c r="I170" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Only an age band is known – a year would be better</t>
         </is>
       </c>
     </row>
@@ -7748,7 +7756,7 @@
       </c>
       <c r="B178" s="5" t="inlineStr">
         <is>
-          <t>B. Sera</t>
+          <t>Ben Sera</t>
         </is>
       </c>
       <c r="C178" s="5" t="inlineStr">
@@ -7756,18 +7764,32 @@
           <t>2017–2022</t>
         </is>
       </c>
-      <c r="D178" s="6" t="inlineStr"/>
-      <c r="E178" s="7" t="n"/>
-      <c r="F178" s="5" t="inlineStr"/>
+      <c r="D178" s="6" t="inlineStr">
+        <is>
+          <t>1988</t>
+        </is>
+      </c>
+      <c r="E178" s="7" t="n">
+        <v>1988</v>
+      </c>
+      <c r="F178" s="5" t="inlineStr">
+        <is>
+          <t>30–39</t>
+        </is>
+      </c>
       <c r="G178" s="5" t="inlineStr">
         <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="H178" s="8" t="inlineStr"/>
+          <t>Approximate</t>
+        </is>
+      </c>
+      <c r="H178" s="8" t="inlineStr">
+        <is>
+          <t>Graduated college 2010 (Tommy Leech)</t>
+        </is>
+      </c>
       <c r="I178" s="8" t="inlineStr">
         <is>
-          <t>Please add</t>
+          <t>Year only, worked out from an age or school year – a real date would be better</t>
         </is>
       </c>
     </row>
@@ -8261,16 +8283,16 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -8286,16 +8308,16 @@
         <v>92</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">

</xml_diff>